<commit_message>
Folder Update before Group Meeting
</commit_message>
<xml_diff>
--- a/1_Literature_Review/2026_CVPR_Paper_StructureAnalysis.xlsx
+++ b/1_Literature_Review/2026_CVPR_Paper_StructureAnalysis.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaiekvoratham/Documents/GitHub/CU_CompEng_Research/1_Literature_Review/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalappsportal-my.sharepoint.com/personal/kullachart_ekvoratham_dentsu_com/Documents/Documents/CU_CompEng_Research/1_Literature_Review/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05F4BEFE-51F2-BF4B-9D2C-F9E80FBDFD94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="13_ncr:1_{05F4BEFE-51F2-BF4B-9D2C-F9E80FBDFD94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD1150B4-7FB0-4F47-AC5C-955CBD354553}"/>
   <bookViews>
-    <workbookView xWindow="40" yWindow="660" windowWidth="29400" windowHeight="16820" xr2:uid="{53629512-B9B3-CC40-9636-ADC52E20098D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{53629512-B9B3-CC40-9636-ADC52E20098D}"/>
   </bookViews>
   <sheets>
     <sheet name="Writing_Structure" sheetId="3" r:id="rId1"/>
-    <sheet name="Lessons_Learnt_from_Reseach" sheetId="5" r:id="rId2"/>
-    <sheet name="Takeaway" sheetId="4" r:id="rId3"/>
-    <sheet name="all" sheetId="2" r:id="rId4"/>
+    <sheet name="Lessons_Learnt" sheetId="6" r:id="rId2"/>
+    <sheet name="Lessons_Learnt_from_Each" sheetId="5" r:id="rId3"/>
+    <sheet name="Takeaway" sheetId="4" r:id="rId4"/>
+    <sheet name="all" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="226">
   <si>
     <t>Core Insight</t>
   </si>
@@ -696,9 +697,6 @@
   </si>
   <si>
     <t>Actionable Advantage</t>
-  </si>
-  <si>
-    <t>CVPR 2026</t>
   </si>
   <si>
     <t>Breakthrough</t>
@@ -841,12 +839,263 @@
   <si>
     <t>Best Practice - Writing Guideline</t>
   </si>
+  <si>
+    <t>Single-image 3D via probabilistic generation + MITL data engine 
+Asymmetric 1.2B/600M model split; tiered human review</t>
+  </si>
+  <si>
+    <t>One-step editing via Optimal-Transport-derived control field	
+n = 1 noise sample; NFE = 1 per stage</t>
+  </si>
+  <si>
+    <t>Core Idea</t>
+  </si>
+  <si>
+    <t>Field-free latents + native PBR for 3D generation 
+16× spatial compression via SC-VAE</t>
+  </si>
+  <si>
+    <t>Pixels-to-actions vision-action foundation model 
+Auto-labeling via on-screen overlay decoding</t>
+  </si>
+  <si>
+    <t>Unified query-based 4D reconstruction (depth, pose, tracking 
+Independent parallel queries + occupancy grid</t>
+  </si>
+  <si>
+    <t>Specific Innovation / Approach</t>
+  </si>
+  <si>
+    <t>Core Takeaway / Insight</t>
+  </si>
+  <si>
+    <t>SAM 3D</t>
+  </si>
+  <si>
+    <t>Shifts 2D-to-3D reconstruction from a deterministic geometric calculation to conditional probabilistic generation.</t>
+  </si>
+  <si>
+    <t>Handles lost geometry (occlusions) naturally instead of patching loss with heuristics.</t>
+  </si>
+  <si>
+    <t>Reframes one-step image editing as a dynamic Optimal Transport distribution-estimation problem.</t>
+  </si>
+  <si>
+    <t>Reveals the issue was a high-energy, erratic naive drift field, not a missing mask.</t>
+  </si>
+  <si>
+    <t>D4RT</t>
+  </si>
+  <si>
+    <t>Shifts 4D reconstruction to an on-demand query-answering system instead of dense per-frame grid decoding.</t>
+  </si>
+  <si>
+    <t>Unifies previously separate processing modules into a single interface.</t>
+  </si>
+  <si>
+    <t>Structured Latents (TRELLIS 2)</t>
+  </si>
+  <si>
+    <t>Shifts 3D representation away from implicit fields toward a native, field-free explicit structure (O-Voxel).</t>
+  </si>
+  <si>
+    <t>Eliminates field-based representation bottlenecks.</t>
+  </si>
+  <si>
+    <t>Uses a Model-in-the-Loop (MITL) process where humans select/align AI proposals; routes hard cases to expert 3D artists.</t>
+  </si>
+  <si>
+    <t>Scaled to ~1M images and 3M+ meshes by assigning humans tasks they excel at.</t>
+  </si>
+  <si>
+    <t>Auto-labels 71,000 hours of gameplay by decoding on-screen controller overlays via template matching + segmentation.</t>
+  </si>
+  <si>
+    <t>Bypasses manual annotation completely while remaining robust to noisy consumer data.</t>
+  </si>
+  <si>
+    <t>Disentangles geometry, texture, and pose using an asymmetric model split (1.2B geometry, 600M texture/refinement).</t>
+  </si>
+  <si>
+    <t>Prevents cross-task interference in complex generative pipelines.</t>
+  </si>
+  <si>
+    <t>Structured Latents</t>
+  </si>
+  <si>
+    <t>Implements a 3-stage pipeline: sparse structure → geometry → material.</t>
+  </si>
+  <si>
+    <t>Stops training instability caused by joint generation.</t>
+  </si>
+  <si>
+    <t>Decouples structure-preserving transport from optional proximal refinement (each a single forward pass).</t>
+  </si>
+  <si>
+    <t>Improves flexibility and modular control during image editing.</t>
+  </si>
+  <si>
+    <t>Decouples space and time at the query interface, keeping queries strictly independent (no inter-query attention).</t>
+  </si>
+  <si>
+    <t>Independent queries generalize significantly better across domain shifts.</t>
+  </si>
+  <si>
+    <t>Theme 4: Efficiency Over Brute-Force</t>
+  </si>
+  <si>
+    <t>Reduces Monte Carlo variance via the temporal-smoothing structure of its Chord Control Field.</t>
+  </si>
+  <si>
+    <t>Leverages independent parallel queries and occupancy-grid tracking.</t>
+  </si>
+  <si>
+    <t>Delivers 100× to 300× speedups over prior art by scaling costs only to requested points.</t>
+  </si>
+  <si>
+    <t>Makes a 4B parameter model trainable, yielding sub-minute generation times.</t>
+  </si>
+  <si>
+    <t>Uses asymmetric model sizing (1.2B vs. 600M) paired with cost-tiered human review workflows.</t>
+  </si>
+  <si>
+    <t>Maximizes compute performance per dollar/parameter.</t>
+  </si>
+  <si>
+    <t>Uses Jensen's inequality to provide formal error bounds and contraction proofs.</t>
+  </si>
+  <si>
+    <t>Mathematically proves why its smoothing operator suppresses truncation error.</t>
+  </si>
+  <si>
+    <t>Conducts dedicated ablations showing inter-query self-attention leads to overfitting/domain shift.</t>
+  </si>
+  <si>
+    <t>Turns an architectural design decision into a generalizable lesson for the field.</t>
+  </si>
+  <si>
+    <t>Gives mathematical rigor to what the model is estimating.</t>
+  </si>
+  <si>
+    <t>Releases SA-3DAO: 1,000 real image–3D pairs curated to a professional artist "human upper bound."</t>
+  </si>
+  <si>
+    <t>Sets a new gold standard for high-quality 3D evaluation.</t>
+  </si>
+  <si>
+    <t>Introduces a universal Gymnasium-style gameplay harness across commercial games.</t>
+  </si>
+  <si>
+    <t>Enables standardized cross-game testing without modifying game source code.</t>
+  </si>
+  <si>
+    <t>Accelerates progress by borrowing mature training regimes.</t>
+  </si>
+  <si>
+    <t>Shifts focus from Vision-Language modeling to Vision-Action modeling on video data.</t>
+  </si>
+  <si>
+    <t>Treats gameplay video with the same methodology as robotics demonstration footage.</t>
+  </si>
+  <si>
+    <t>Replaces standard CNN residual blocks with Transformer-style wide pointwise MLPs inside the VAE.</t>
+  </si>
+  <si>
+    <t>Modernizes standard VAE building blocks for superior representation.</t>
+  </si>
+  <si>
+    <t>Theme 8: Honest Limitations</t>
+  </si>
+  <si>
+    <t>Transparently details dataset noise (UI lag/artifacts) and its System-1 nature (no long-horizon planning).</t>
+  </si>
+  <si>
+    <t>Frames noise handling as proof of model robustness while outlining clear VLA future work.</t>
+  </si>
+  <si>
+    <t>Explicitly acknowledges fundamental information loss during 2D-to-3D inversion.</t>
+  </si>
+  <si>
+    <t>Directly justifies the necessity of its probabilistic approach.</t>
+  </si>
+  <si>
+    <t>Theme 1: Reframe the Problem 
+(Change what is computed rather than tuning old heuristics)</t>
+  </si>
+  <si>
+    <t>Theme 2: Solve the Data Bottleneck 
+(Treat data synthesis and labeling as first-class research)</t>
+  </si>
+  <si>
+    <t>SC-VAE delivers 16× spatial compression (1024^3 &gt; 9.6 tokens).</t>
+  </si>
+  <si>
+    <t>Achieves seed-robustness using a single noise sample (n = 1).</t>
+  </si>
+  <si>
+    <t>Defines a formal probabilistic notation Pr(S,T,R,t,s |I,M).</t>
+  </si>
+  <si>
+    <t>Applies the LLM training lifecycle (pretrain &gt; mid-train &gt; post-train) to 3D.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theme 3: Decouple &amp; Modularize Systems </t>
+  </si>
+  <si>
+    <t>Split complex targets into independent sub-components</t>
+  </si>
+  <si>
+    <t>Theme</t>
+  </si>
+  <si>
+    <t>Prioritize smart compute allocation over parameter scaling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theme 5: Ground Wins in Theory </t>
+  </si>
+  <si>
+    <t>Provide formal proofs and ablations explaining WHY it works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theme 6: Build the Benchmark </t>
+  </si>
+  <si>
+    <t>Create evaluation infrastructure to guide future research</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theme 7: Cross-Domain Paradigms </t>
+  </si>
+  <si>
+    <t>Import proven recipes from one modality into another</t>
+  </si>
+  <si>
+    <t>Acknowledge weaknesses transparently to build trust</t>
+  </si>
+  <si>
+    <t>Brief</t>
+  </si>
+  <si>
+    <t>A generative foundation model designed to reconstruct high-quality 3D geometry, texture, and spatial layout from just a single real-world image, even in complex or heavily occluded environments
+To overcome the historical "data barrier" in 3D AI, the researchers developed a Model-in-the-Loop (MITL) data engine that scales human-vetted annotations by having AI generate initial proposals for human curation and professional artist refinement.</t>
+  </si>
+  <si>
+    <t>ChordEdit introduces a training-free, inversion-free image editing framework designed to overcome the structural instability and background corruption common in fast, single-step generative models. By replacing naive drift tracking with a mathematically constrained Chord Control Field, the algorithm smooths high-energy velocity spikes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduce the representation that natively encodes both complex 3D geometry and physically-based rendering (PBR) material properties, allowing instant, optimization-free conversions between raw meshes and neural latents. </t>
+  </si>
+  <si>
+    <t>An open-source foundation model designed for video game environments that addresses the scarcity of action-labeled training data by automatically extracting player inputs from over 40,000 hours of public gameplay videos featuring on-screen gamepad overlays.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instead of relying on slow, complex pipelines with task-specific decoders or per-frame dense decoding, D4RT encodes the input video into a global scene representation and uses a lightweight cross-attention decoder to independently query the 3D position of any point at any space and time coordinate. </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -932,8 +1181,47 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -946,8 +1234,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1035,11 +1341,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1104,14 +1462,71 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1616,38 +2031,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCE6C4E3-585C-EE4B-9259-53D9E4658DCF}">
   <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="30.83203125" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="30.83203125" defaultRowHeight="14" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="3.1640625" style="20" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" style="11" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" style="11" customWidth="1"/>
-    <col min="4" max="4" width="70.83203125" style="11" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" style="32" customWidth="1"/>
+    <col min="4" max="4" width="65.58203125" style="11" customWidth="1"/>
     <col min="5" max="5" width="30.83203125" style="11" customWidth="1"/>
     <col min="6" max="16384" width="30.83203125" style="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="B1" s="19" t="s">
+    <row r="1" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="B1" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="E1" s="19" t="s">
+      <c r="D1" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="34" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="120" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="126" x14ac:dyDescent="0.4">
       <c r="A2" s="20">
         <v>1</v>
       </c>
       <c r="B2" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="32" t="s">
         <v>57</v>
       </c>
       <c r="D2" s="11" t="s">
@@ -1657,14 +2072,14 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="112" x14ac:dyDescent="0.4">
       <c r="A3" s="20">
         <v>2</v>
       </c>
       <c r="B3" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="32" t="s">
         <v>59</v>
       </c>
       <c r="D3" s="11" t="s">
@@ -1674,14 +2089,14 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="120" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="112" x14ac:dyDescent="0.4">
       <c r="A4" s="20">
         <v>3</v>
       </c>
       <c r="B4" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="32" t="s">
         <v>61</v>
       </c>
       <c r="D4" s="11" t="s">
@@ -1691,14 +2106,14 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="98" x14ac:dyDescent="0.4">
       <c r="A5" s="20">
         <v>4</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="32" t="s">
         <v>63</v>
       </c>
       <c r="D5" s="11" t="s">
@@ -1708,14 +2123,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="90" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="84" x14ac:dyDescent="0.4">
       <c r="A6" s="20">
         <v>5</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="32" t="s">
         <v>66</v>
       </c>
       <c r="D6" s="11" t="s">
@@ -1725,14 +2140,14 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="90" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="84" x14ac:dyDescent="0.4">
       <c r="A7" s="20">
         <v>6</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="32" t="s">
         <v>68</v>
       </c>
       <c r="D7" s="11" t="s">
@@ -1742,14 +2157,14 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="98" x14ac:dyDescent="0.4">
       <c r="A8" s="20">
         <v>7</v>
       </c>
       <c r="B8" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="32" t="s">
         <v>71</v>
       </c>
       <c r="D8" s="11" t="s">
@@ -1759,14 +2174,14 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="98" x14ac:dyDescent="0.4">
       <c r="A9" s="20">
         <v>8</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="32" t="s">
         <v>72</v>
       </c>
       <c r="D9" s="11" t="s">
@@ -1776,14 +2191,14 @@
         <v>73</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="105" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="98" x14ac:dyDescent="0.4">
       <c r="A10" s="20">
         <v>9</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="32" t="s">
         <v>75</v>
       </c>
       <c r="D10" s="11" t="s">
@@ -1793,14 +2208,14 @@
         <v>93</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="70" x14ac:dyDescent="0.4">
       <c r="A11" s="20">
         <v>10</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="32" t="s">
         <v>77</v>
       </c>
       <c r="D11" s="11" t="s">
@@ -1810,14 +2225,14 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="84" x14ac:dyDescent="0.4">
       <c r="A12" s="20">
         <v>11</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="32" t="s">
         <v>79</v>
       </c>
       <c r="D12" s="11" t="s">
@@ -1833,105 +2248,531 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{400DF996-A38F-E643-AFF1-8C2BF0CAD0C0}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="30.83203125" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84289E5D-6587-4B0C-BABF-129F44549B8B}">
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr defaultColWidth="30.58203125" defaultRowHeight="12.5" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" style="19" customWidth="1"/>
-    <col min="2" max="4" width="40.83203125" style="11" customWidth="1"/>
-    <col min="5" max="16384" width="30.83203125" style="11"/>
+    <col min="1" max="1" width="20.58203125" style="27" customWidth="1"/>
+    <col min="2" max="2" width="15.58203125" style="31" customWidth="1"/>
+    <col min="3" max="3" width="20.58203125" style="24" customWidth="1"/>
+    <col min="4" max="16384" width="30.58203125" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:5" s="30" customFormat="1" ht="13" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="28" t="s">
+        <v>211</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>151</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="38" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" s="41" t="s">
+        <v>203</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="40"/>
+      <c r="B3" s="42"/>
+      <c r="C3" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="50.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="40"/>
+      <c r="B4" s="42"/>
+      <c r="C4" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="39"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="B6" s="41" t="s">
+        <v>204</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="50.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="39"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="B8" s="41" t="s">
+        <v>210</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="25.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="40"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>171</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="50.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="40"/>
+      <c r="B10" s="42"/>
+      <c r="C10" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>173</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="50.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="39"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>175</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="38" t="s">
+        <v>177</v>
+      </c>
+      <c r="B12" s="41" t="s">
+        <v>212</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="E12" s="26" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="40"/>
+      <c r="B13" s="42"/>
+      <c r="C13" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>179</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="40"/>
+      <c r="B14" s="42"/>
+      <c r="C14" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>205</v>
+      </c>
+      <c r="E14" s="25" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="39"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>182</v>
+      </c>
+      <c r="E15" s="25" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="50.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="38" t="s">
+        <v>213</v>
+      </c>
+      <c r="B16" s="41" t="s">
+        <v>214</v>
+      </c>
+      <c r="C16" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="E16" s="26" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="40"/>
+      <c r="B17" s="42"/>
+      <c r="C17" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>186</v>
+      </c>
+      <c r="E17" s="25" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="25.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="39"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>207</v>
+      </c>
+      <c r="E18" s="25" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="50.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="B19" s="41" t="s">
+        <v>216</v>
+      </c>
+      <c r="C19" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="D19" s="26" t="s">
+        <v>189</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="39"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="E20" s="25" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="50.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="38" t="s">
+        <v>217</v>
+      </c>
+      <c r="B21" s="41" t="s">
+        <v>218</v>
+      </c>
+      <c r="C21" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="D21" s="26" t="s">
+        <v>208</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="40"/>
+      <c r="B22" s="42"/>
+      <c r="C22" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>194</v>
+      </c>
+      <c r="E22" s="25" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="39"/>
+      <c r="B23" s="43"/>
+      <c r="C23" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>196</v>
+      </c>
+      <c r="E23" s="25" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A24" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="B24" s="41" t="s">
+        <v>219</v>
+      </c>
+      <c r="C24" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="D24" s="26" t="s">
+        <v>199</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="38" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="39"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="E25" s="25" t="s">
+        <v>202</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="B16:B18"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{400DF996-A38F-E643-AFF1-8C2BF0CAD0C0}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultColWidth="30.83203125" defaultRowHeight="14" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="15.58203125" style="19" customWidth="1"/>
+    <col min="2" max="2" width="20.58203125" style="11" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" style="11" customWidth="1"/>
+    <col min="4" max="6" width="40.83203125" style="11" customWidth="1"/>
+    <col min="7" max="16384" width="30.83203125" style="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="37" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="35" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>220</v>
+      </c>
+      <c r="D1" s="36" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
-        <v>122</v>
+      <c r="E1" s="36" t="s">
+        <v>123</v>
+      </c>
+      <c r="F1" s="36" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="196" x14ac:dyDescent="0.4">
+      <c r="A2" s="23" t="s">
+        <v>126</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>123</v>
+        <v>221</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="135" x14ac:dyDescent="0.2">
-      <c r="A3" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="140" x14ac:dyDescent="0.4">
+      <c r="A3" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>222</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="112" x14ac:dyDescent="0.4">
+      <c r="A4" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="B3" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="D3" s="23" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="135" x14ac:dyDescent="0.2">
-      <c r="A4" s="24" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="D4" s="23" t="s">
+      <c r="B4" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>223</v>
+      </c>
+      <c r="D4" s="22" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="135" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+      <c r="E4" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="140" x14ac:dyDescent="0.4">
+      <c r="A5" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>224</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="126" x14ac:dyDescent="0.4">
+      <c r="A6" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="B5" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>137</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="150" x14ac:dyDescent="0.2">
-      <c r="A6" s="24" t="s">
-        <v>121</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="C6" s="23" t="s">
+      <c r="B6" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="D6" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D6" s="23" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="135" x14ac:dyDescent="0.2">
-      <c r="A7" s="24" t="s">
-        <v>129</v>
-      </c>
-      <c r="B7" s="23" t="s">
+      <c r="E6" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="F6" s="22" t="s">
         <v>142</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -1939,10 +2780,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B42CFC8-D437-CB44-86D8-0FCCC6CDC72C}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="40.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="40.83203125" defaultRowHeight="14.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="3.1640625" style="21" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" style="21" customWidth="1"/>
@@ -1950,7 +2791,7 @@
     <col min="4" max="16384" width="40.83203125" style="21"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="B1" s="19" t="s">
         <v>81</v>
       </c>
@@ -1958,7 +2799,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="42" x14ac:dyDescent="0.4">
       <c r="A2" s="21">
         <v>1</v>
       </c>
@@ -1969,7 +2810,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="42" x14ac:dyDescent="0.4">
       <c r="A3" s="21">
         <v>2</v>
       </c>
@@ -1980,7 +2821,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="42" x14ac:dyDescent="0.4">
       <c r="A4" s="21">
         <v>3</v>
       </c>
@@ -1991,7 +2832,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="42" x14ac:dyDescent="0.4">
       <c r="A5" s="21">
         <v>4</v>
       </c>
@@ -2002,7 +2843,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="60" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="56" x14ac:dyDescent="0.4">
       <c r="A6" s="21">
         <v>5</v>
       </c>
@@ -2013,7 +2854,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="42" x14ac:dyDescent="0.4">
       <c r="A7" s="21">
         <v>6</v>
       </c>
@@ -2024,7 +2865,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="28" x14ac:dyDescent="0.4">
       <c r="A8" s="21">
         <v>7</v>
       </c>
@@ -2035,7 +2876,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="42" x14ac:dyDescent="0.4">
       <c r="A9" s="21">
         <v>8</v>
       </c>
@@ -2046,7 +2887,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="42" x14ac:dyDescent="0.4">
       <c r="A10" s="21">
         <v>9</v>
       </c>
@@ -2057,7 +2898,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="45" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="42" x14ac:dyDescent="0.4">
       <c r="A11" s="21">
         <v>10</v>
       </c>
@@ -2073,10 +2914,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5AE4AD9-CDC6-6244-AD27-653FDC5D6AAB}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="30.83203125" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="30.83203125" defaultRowHeight="14" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="2.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="20.83203125" style="11" customWidth="1"/>
@@ -2086,7 +2927,7 @@
     <col min="7" max="16384" width="30.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="19" customFormat="1" ht="30" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="19" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="17"/>
       <c r="B1" s="13" t="s">
         <v>54</v>
@@ -2104,7 +2945,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="332" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="287.5" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2124,7 +2965,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="375" x14ac:dyDescent="0.4">
       <c r="A3" s="5">
         <f>A2+1</f>
         <v>2</v>
@@ -2145,7 +2986,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="409.5" x14ac:dyDescent="0.4">
       <c r="A4" s="5">
         <f t="shared" ref="A4:A12" si="0">A3+1</f>
         <v>3</v>
@@ -2166,7 +3007,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="375" x14ac:dyDescent="0.4">
       <c r="A5" s="5">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2187,7 +3028,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="306" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="275" x14ac:dyDescent="0.4">
       <c r="A6" s="5">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2208,7 +3049,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="350" x14ac:dyDescent="0.4">
       <c r="A7" s="5">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2229,7 +3070,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="345" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="312.5" x14ac:dyDescent="0.4">
       <c r="A8" s="5">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2250,7 +3091,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="280" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="250" x14ac:dyDescent="0.4">
       <c r="A9" s="5">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2271,7 +3112,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="362.5" x14ac:dyDescent="0.4">
       <c r="A10" s="5">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2292,7 +3133,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="362.5" x14ac:dyDescent="0.4">
       <c r="A11" s="5">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2313,7 +3154,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="409.5" x14ac:dyDescent="0.4">
       <c r="A12" s="5">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2340,4 +3181,10 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{6e8992ec-76d5-4ea5-8eae-b0c5e558749a}" enabled="0" method="" siteId="{6e8992ec-76d5-4ea5-8eae-b0c5e558749a}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>